<commit_message>
docs: add 14 new native commands to commands framework
</commit_message>
<xml_diff>
--- a/docs/process/commands_framework.xlsx
+++ b/docs/process/commands_framework.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +44,12 @@
       <color rgb="00555555"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +86,11 @@
         <fgColor rgb="00D6E8FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -109,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -134,6 +143,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -500,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2235,6 +2247,594 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Dados / Análise</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>/xlsx</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Gera e edita planilhas Excel com formatação e fórmulas</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>Relatórios financeiros, tabelas de dados, frameworks</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>"Crie um Excel com métricas do projeto" → gera e salva o .xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>Dados / Análise</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>/validate-data</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>Valida qualidade e consistência de datasets</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>Antes de usar dados em análise ou modelo</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>"Valide esse CSV antes de processar" → reporta erros e anomalias</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>Dados / Análise</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>/write-query</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Escreve queries SQL ou equivalentes a partir de linguagem natural</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>Extração de dados, análise exploratória</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
+        <is>
+          <t>"Quero os deputados com mais de 10 faltas" → gera a query</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>Produto / Eng</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>/write-spec</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>Escreve especificações técnicas ou de produto</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>Antes de implementar uma feature</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
+        <is>
+          <t>"Escreva a spec para o módulo de alertas" → gera documento estruturado</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>UX / Research</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>/ux-copy</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>Escreve e refina microcopy, textos de UI e comunicação com usuário</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>Botões, mensagens de erro, onboarding, tooltips</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>"Escreva o texto do botão de confirmação e da mensagem de erro" → gera variações</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>Processo</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>/wizard</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Nativo (só no template pai)</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>Setup guiado de um novo projeto a partir do template</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>Inicializar repositório novo com o template</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
+        <is>
+          <t>"Novo projeto" → wizard pergunta nome, owner, stack e configura tudo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>Processo</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>/ultrareview</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>Code review aprofundado com análise de segurança, performance e design</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>PRs críticos, revisão pré-release</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>"Rode ultrareview no PR #42" → análise detalhada além do /review padrão</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>Processo</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>/schedule</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>Agenda tarefas recorrentes ou com delay</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Automações periódicas, lembretes</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
+        <is>
+          <t>"Rode /standup todo dia às 9h" → cria cron no Claude Code</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Processo</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>/rewind</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>Reverte o contexto da sessão para um ponto anterior</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Desfazer ações indesejadas na sessão</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
+        <is>
+          <t>"Volte antes da última edição" → restaura estado anterior</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>/btw</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Adiciona contexto lateral sem interromper o fluxo principal</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>Notas rápidas, avisos ao Claude sem mudar tarefa</t>
+        </is>
+      </c>
+      <c r="H51" s="9" t="inlineStr">
+        <is>
+          <t>"btw: não use print, use logging" → Claude incorpora sem parar o que fazia</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>/mcp</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>Gerencia MCP servers conectados ao Claude Code</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>Listar, adicionar ou remover MCPs</t>
+        </is>
+      </c>
+      <c r="H52" s="9" t="inlineStr">
+        <is>
+          <t>"Liste os MCPs ativos" → mostra conexões disponíveis</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>/model</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Troca o modelo Claude em uso na sessão</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>Usar Opus para tarefas complexas, Haiku para rápidas</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>"Mude para claude-opus-4-7" → troca o modelo sem reiniciar</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>/clear</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>Limpa o contexto da conversa atual</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>Reiniciar sessão sem fechar o terminal</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>"Limpe o contexto" → nova conversa em branco</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>/export</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Nativo</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Exporta o conteúdo da sessão atual</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>Salvar conversa, compartilhar resultado</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>"Exporte essa sessão" → gera arquivo com o histórico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>